<commit_message>
Map county misspellings and alternate signals in extract_county
Add COUNTY_ALIASES (Altantic -> Atlantic, Monmout -> Monmouth,
Newark -> Essex) to the notebook's extract_county. Aliases join the
county regex and every match is mapped back to its county via a
lookup map. Add alias spot checks, and relabel the 10 spreadsheet
rows the aliases now resolve.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RJZUYzMR2Vofw2PSUEVq2i
</commit_message>
<xml_diff>
--- a/tests/missing_program_county_sql_338.xlsx
+++ b/tests/missing_program_county_sql_338.xlsx
@@ -1610,7 +1610,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Essex</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -4790,7 +4790,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Essex</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
@@ -9180,7 +9180,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Essex</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -9209,7 +9209,7 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Essex</t>
         </is>
       </c>
       <c r="L145" t="inlineStr">
@@ -9628,7 +9628,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -9657,7 +9657,7 @@
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="L152" t="inlineStr">
@@ -9692,7 +9692,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Essex</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
@@ -9721,7 +9721,7 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Essex</t>
         </is>
       </c>
       <c r="L153" t="inlineStr">
@@ -10972,7 +10972,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Monmouth</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
@@ -11006,7 +11006,7 @@
       </c>
       <c r="L173" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Monmouth</t>
         </is>
       </c>
       <c r="M173" t="inlineStr">
@@ -14812,7 +14812,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Monmouth</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
@@ -14846,7 +14846,7 @@
       </c>
       <c r="L233" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Monmouth</t>
         </is>
       </c>
       <c r="M233" t="inlineStr">
@@ -16540,7 +16540,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Monmouth</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
@@ -16574,7 +16574,7 @@
       </c>
       <c r="L260" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Monmouth</t>
         </is>
       </c>
       <c r="M260" t="inlineStr">
@@ -16860,7 +16860,7 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Monmouth</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
@@ -16894,7 +16894,7 @@
       </c>
       <c r="L265" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Monmouth</t>
         </is>
       </c>
       <c r="M265" t="inlineStr">
@@ -19996,7 +19996,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Monmouth</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -20030,7 +20030,7 @@
       </c>
       <c r="L314" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Monmouth</t>
         </is>
       </c>
       <c r="M314" t="inlineStr">

</xml_diff>